<commit_message>
Integrate MGCECDL inference workflow
</commit_message>
<xml_diff>
--- a/data/Variables_seleccion.xlsx
+++ b/data/Variables_seleccion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Documents/CHEC/chec_impacto/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E1BD558-52A2-CC48-99E9-C6646785D5C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169BF0B5-BF74-2F45-A337-BAC10B79FE72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables_análisis" sheetId="1" r:id="rId1"/>
@@ -712,7 +712,7 @@
         <v>20</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -1196,7 +1196,7 @@
         <v>108</v>
       </c>
       <c r="C54">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="16" x14ac:dyDescent="0.25">

</xml_diff>